<commit_message>
v9.6.1: address Codex review (atomic lockout, AUTH_USERS precedence, /__me detection, xlsx sheet choice, share limits, board restore, modified samples)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NrcW6JZnHC5gGLR7krQk3
</commit_message>
<xml_diff>
--- a/tests/fixtures/spi-sample.xlsx
+++ b/tests/fixtures/spi-sample.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,13 +418,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>這張工作表只有說明</t>
+          <t>欄位說明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Board：板號</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Volume：體積 %</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>必填</t>
         </is>
       </c>
     </row>
@@ -530,7 +554,7 @@
       <c r="I2" t="n">
         <v>-14</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -570,7 +594,7 @@
       <c r="I3" t="n">
         <v>3.7</v>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -610,7 +634,7 @@
       <c r="I4" t="n">
         <v>7.6</v>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -650,7 +674,7 @@
       <c r="I5" t="n">
         <v>-7</v>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -690,7 +714,7 @@
       <c r="I6" t="n">
         <v>4.6</v>
       </c>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -730,7 +754,7 @@
       <c r="I7" t="n">
         <v>18</v>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -770,7 +794,7 @@
       <c r="I8" t="n">
         <v>9.5</v>
       </c>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -810,7 +834,7 @@
       <c r="I9" t="n">
         <v>18.3</v>
       </c>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -850,7 +874,7 @@
       <c r="I10" t="n">
         <v>0.7</v>
       </c>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -890,7 +914,7 @@
       <c r="I11" t="n">
         <v>-12.3</v>
       </c>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -930,7 +954,7 @@
       <c r="I12" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -970,7 +994,7 @@
       <c r="I13" t="n">
         <v>-19.5</v>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1010,7 +1034,7 @@
       <c r="I14" t="n">
         <v>-14.5</v>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1050,7 +1074,7 @@
       <c r="I15" t="n">
         <v>3.6</v>
       </c>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1090,7 +1114,7 @@
       <c r="I16" t="n">
         <v>5.4</v>
       </c>
-      <c r="J16" s="1" t="n">
+      <c r="J16" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1130,7 +1154,7 @@
       <c r="I17" t="n">
         <v>2.4</v>
       </c>
-      <c r="J17" s="1" t="n">
+      <c r="J17" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1170,7 +1194,7 @@
       <c r="I18" t="n">
         <v>7.8</v>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1210,7 +1234,7 @@
       <c r="I19" t="n">
         <v>7.9</v>
       </c>
-      <c r="J19" s="1" t="n">
+      <c r="J19" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1250,7 +1274,7 @@
       <c r="I20" t="n">
         <v>-2.8</v>
       </c>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1290,7 +1314,7 @@
       <c r="I21" t="n">
         <v>-2.3</v>
       </c>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>46296.33541666667</v>
       </c>
     </row>
@@ -1330,7 +1354,7 @@
       <c r="I22" t="n">
         <v>-9.9</v>
       </c>
-      <c r="J22" s="1" t="n">
+      <c r="J22" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1370,7 +1394,7 @@
       <c r="I23" t="n">
         <v>14.2</v>
       </c>
-      <c r="J23" s="1" t="n">
+      <c r="J23" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1410,7 +1434,7 @@
       <c r="I24" t="n">
         <v>-2.2</v>
       </c>
-      <c r="J24" s="1" t="n">
+      <c r="J24" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1450,7 +1474,7 @@
       <c r="I25" t="n">
         <v>-19</v>
       </c>
-      <c r="J25" s="1" t="n">
+      <c r="J25" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1490,7 +1514,7 @@
       <c r="I26" t="n">
         <v>5.2</v>
       </c>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1530,7 +1554,7 @@
       <c r="I27" t="n">
         <v>4.2</v>
       </c>
-      <c r="J27" s="1" t="n">
+      <c r="J27" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1570,7 +1594,7 @@
       <c r="I28" t="n">
         <v>30.2</v>
       </c>
-      <c r="J28" s="1" t="n">
+      <c r="J28" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1610,7 +1634,7 @@
       <c r="I29" t="n">
         <v>13.9</v>
       </c>
-      <c r="J29" s="1" t="n">
+      <c r="J29" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1650,7 +1674,7 @@
       <c r="I30" t="n">
         <v>-16.9</v>
       </c>
-      <c r="J30" s="1" t="n">
+      <c r="J30" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1690,7 +1714,7 @@
       <c r="I31" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1730,7 +1754,7 @@
       <c r="I32" t="n">
         <v>-8.300000000000001</v>
       </c>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1770,7 +1794,7 @@
       <c r="I33" t="n">
         <v>-7.3</v>
       </c>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1810,7 +1834,7 @@
       <c r="I34" t="n">
         <v>12.8</v>
       </c>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1850,7 +1874,7 @@
       <c r="I35" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1890,7 +1914,7 @@
       <c r="I36" t="n">
         <v>10.2</v>
       </c>
-      <c r="J36" s="1" t="n">
+      <c r="J36" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1930,7 +1954,7 @@
       <c r="I37" t="n">
         <v>2.9</v>
       </c>
-      <c r="J37" s="1" t="n">
+      <c r="J37" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -1970,7 +1994,7 @@
       <c r="I38" t="n">
         <v>15.7</v>
       </c>
-      <c r="J38" s="1" t="n">
+      <c r="J38" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -2010,7 +2034,7 @@
       <c r="I39" t="n">
         <v>-4</v>
       </c>
-      <c r="J39" s="1" t="n">
+      <c r="J39" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -2050,7 +2074,7 @@
       <c r="I40" t="n">
         <v>-22.9</v>
       </c>
-      <c r="J40" s="1" t="n">
+      <c r="J40" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -2090,7 +2114,7 @@
       <c r="I41" t="n">
         <v>-22.1</v>
       </c>
-      <c r="J41" s="1" t="n">
+      <c r="J41" s="2" t="n">
         <v>46296.3375</v>
       </c>
     </row>
@@ -2130,7 +2154,7 @@
       <c r="I42" t="n">
         <v>0</v>
       </c>
-      <c r="J42" s="1" t="n">
+      <c r="J42" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2170,7 +2194,7 @@
       <c r="I43" t="n">
         <v>23.4</v>
       </c>
-      <c r="J43" s="1" t="n">
+      <c r="J43" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2210,7 +2234,7 @@
       <c r="I44" t="n">
         <v>-1.4</v>
       </c>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2250,7 +2274,7 @@
       <c r="I45" t="n">
         <v>-15.3</v>
       </c>
-      <c r="J45" s="1" t="n">
+      <c r="J45" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2290,7 +2314,7 @@
       <c r="I46" t="n">
         <v>-11.2</v>
       </c>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2330,7 +2354,7 @@
       <c r="I47" t="n">
         <v>-4</v>
       </c>
-      <c r="J47" s="1" t="n">
+      <c r="J47" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2370,7 +2394,7 @@
       <c r="I48" t="n">
         <v>4.8</v>
       </c>
-      <c r="J48" s="1" t="n">
+      <c r="J48" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2410,7 +2434,7 @@
       <c r="I49" t="n">
         <v>19.9</v>
       </c>
-      <c r="J49" s="1" t="n">
+      <c r="J49" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2450,7 +2474,7 @@
       <c r="I50" t="n">
         <v>-10.1</v>
       </c>
-      <c r="J50" s="1" t="n">
+      <c r="J50" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2490,7 +2514,7 @@
       <c r="I51" t="n">
         <v>16</v>
       </c>
-      <c r="J51" s="1" t="n">
+      <c r="J51" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2530,7 +2554,7 @@
       <c r="I52" t="n">
         <v>-8.9</v>
       </c>
-      <c r="J52" s="1" t="n">
+      <c r="J52" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2570,7 +2594,7 @@
       <c r="I53" t="n">
         <v>15</v>
       </c>
-      <c r="J53" s="1" t="n">
+      <c r="J53" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2610,7 +2634,7 @@
       <c r="I54" t="n">
         <v>-24.7</v>
       </c>
-      <c r="J54" s="1" t="n">
+      <c r="J54" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2650,7 +2674,7 @@
       <c r="I55" t="n">
         <v>12.1</v>
       </c>
-      <c r="J55" s="1" t="n">
+      <c r="J55" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2690,7 +2714,7 @@
       <c r="I56" t="n">
         <v>13.8</v>
       </c>
-      <c r="J56" s="1" t="n">
+      <c r="J56" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2730,7 +2754,7 @@
       <c r="I57" t="n">
         <v>-1.8</v>
       </c>
-      <c r="J57" s="1" t="n">
+      <c r="J57" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2770,7 +2794,7 @@
       <c r="I58" t="n">
         <v>-9.6</v>
       </c>
-      <c r="J58" s="1" t="n">
+      <c r="J58" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2810,7 +2834,7 @@
       <c r="I59" t="n">
         <v>-13.1</v>
       </c>
-      <c r="J59" s="1" t="n">
+      <c r="J59" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2850,7 +2874,7 @@
       <c r="I60" t="n">
         <v>10</v>
       </c>
-      <c r="J60" s="1" t="n">
+      <c r="J60" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2890,7 +2914,7 @@
       <c r="I61" t="n">
         <v>-31.3</v>
       </c>
-      <c r="J61" s="1" t="n">
+      <c r="J61" s="2" t="n">
         <v>46296.33958333333</v>
       </c>
     </row>
@@ -2930,7 +2954,7 @@
       <c r="I62" t="n">
         <v>29.1</v>
       </c>
-      <c r="J62" s="1" t="n">
+      <c r="J62" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -2970,7 +2994,7 @@
       <c r="I63" t="n">
         <v>10.3</v>
       </c>
-      <c r="J63" s="1" t="n">
+      <c r="J63" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3010,7 +3034,7 @@
       <c r="I64" t="n">
         <v>-13.6</v>
       </c>
-      <c r="J64" s="1" t="n">
+      <c r="J64" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3050,7 +3074,7 @@
       <c r="I65" t="n">
         <v>-2.9</v>
       </c>
-      <c r="J65" s="1" t="n">
+      <c r="J65" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3090,7 +3114,7 @@
       <c r="I66" t="n">
         <v>-12.8</v>
       </c>
-      <c r="J66" s="1" t="n">
+      <c r="J66" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3130,7 +3154,7 @@
       <c r="I67" t="n">
         <v>-38.9</v>
       </c>
-      <c r="J67" s="1" t="n">
+      <c r="J67" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3170,7 +3194,7 @@
       <c r="I68" t="n">
         <v>-1</v>
       </c>
-      <c r="J68" s="1" t="n">
+      <c r="J68" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3210,7 +3234,7 @@
       <c r="I69" t="n">
         <v>-10.5</v>
       </c>
-      <c r="J69" s="1" t="n">
+      <c r="J69" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3250,7 +3274,7 @@
       <c r="I70" t="n">
         <v>4.4</v>
       </c>
-      <c r="J70" s="1" t="n">
+      <c r="J70" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3290,7 +3314,7 @@
       <c r="I71" t="n">
         <v>15.6</v>
       </c>
-      <c r="J71" s="1" t="n">
+      <c r="J71" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3330,7 +3354,7 @@
       <c r="I72" t="n">
         <v>27.3</v>
       </c>
-      <c r="J72" s="1" t="n">
+      <c r="J72" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3370,7 +3394,7 @@
       <c r="I73" t="n">
         <v>-11.2</v>
       </c>
-      <c r="J73" s="1" t="n">
+      <c r="J73" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3410,7 +3434,7 @@
       <c r="I74" t="n">
         <v>6.9</v>
       </c>
-      <c r="J74" s="1" t="n">
+      <c r="J74" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3450,7 +3474,7 @@
       <c r="I75" t="n">
         <v>11.8</v>
       </c>
-      <c r="J75" s="1" t="n">
+      <c r="J75" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3485,12 +3509,12 @@
         <v>92.90000000000001</v>
       </c>
       <c r="H76" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I76" t="n">
         <v>-1.6</v>
       </c>
-      <c r="J76" s="1" t="n">
+      <c r="J76" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3530,7 +3554,7 @@
       <c r="I77" t="n">
         <v>-18.9</v>
       </c>
-      <c r="J77" s="1" t="n">
+      <c r="J77" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3570,7 +3594,7 @@
       <c r="I78" t="n">
         <v>6.7</v>
       </c>
-      <c r="J78" s="1" t="n">
+      <c r="J78" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3610,7 +3634,7 @@
       <c r="I79" t="n">
         <v>11.1</v>
       </c>
-      <c r="J79" s="1" t="n">
+      <c r="J79" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3650,7 +3674,7 @@
       <c r="I80" t="n">
         <v>-5.7</v>
       </c>
-      <c r="J80" s="1" t="n">
+      <c r="J80" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3690,7 +3714,7 @@
       <c r="I81" t="n">
         <v>2.7</v>
       </c>
-      <c r="J81" s="1" t="n">
+      <c r="J81" s="2" t="n">
         <v>46296.34166666667</v>
       </c>
     </row>
@@ -3730,7 +3754,7 @@
       <c r="I82" t="n">
         <v>24.8</v>
       </c>
-      <c r="J82" s="1" t="n">
+      <c r="J82" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -3770,7 +3794,7 @@
       <c r="I83" t="n">
         <v>10.9</v>
       </c>
-      <c r="J83" s="1" t="n">
+      <c r="J83" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -3810,7 +3834,7 @@
       <c r="I84" t="n">
         <v>-3.2</v>
       </c>
-      <c r="J84" s="1" t="n">
+      <c r="J84" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -3850,7 +3874,7 @@
       <c r="I85" t="n">
         <v>38.9</v>
       </c>
-      <c r="J85" s="1" t="n">
+      <c r="J85" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -3890,7 +3914,7 @@
       <c r="I86" t="n">
         <v>-17.5</v>
       </c>
-      <c r="J86" s="1" t="n">
+      <c r="J86" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -3930,7 +3954,7 @@
       <c r="I87" t="n">
         <v>0.4</v>
       </c>
-      <c r="J87" s="1" t="n">
+      <c r="J87" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -3970,7 +3994,7 @@
       <c r="I88" t="n">
         <v>-3.7</v>
       </c>
-      <c r="J88" s="1" t="n">
+      <c r="J88" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4010,7 +4034,7 @@
       <c r="I89" t="n">
         <v>-22</v>
       </c>
-      <c r="J89" s="1" t="n">
+      <c r="J89" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4050,7 +4074,7 @@
       <c r="I90" t="n">
         <v>8.5</v>
       </c>
-      <c r="J90" s="1" t="n">
+      <c r="J90" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4090,7 +4114,7 @@
       <c r="I91" t="n">
         <v>7.7</v>
       </c>
-      <c r="J91" s="1" t="n">
+      <c r="J91" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4130,7 +4154,7 @@
       <c r="I92" t="n">
         <v>11.7</v>
       </c>
-      <c r="J92" s="1" t="n">
+      <c r="J92" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4170,7 +4194,7 @@
       <c r="I93" t="n">
         <v>-26.4</v>
       </c>
-      <c r="J93" s="1" t="n">
+      <c r="J93" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4210,7 +4234,7 @@
       <c r="I94" t="n">
         <v>0.5</v>
       </c>
-      <c r="J94" s="1" t="n">
+      <c r="J94" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4250,7 +4274,7 @@
       <c r="I95" t="n">
         <v>17.5</v>
       </c>
-      <c r="J95" s="1" t="n">
+      <c r="J95" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4290,7 +4314,7 @@
       <c r="I96" t="n">
         <v>-1.2</v>
       </c>
-      <c r="J96" s="1" t="n">
+      <c r="J96" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4330,7 +4354,7 @@
       <c r="I97" t="n">
         <v>-0.3</v>
       </c>
-      <c r="J97" s="1" t="n">
+      <c r="J97" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4370,7 +4394,7 @@
       <c r="I98" t="n">
         <v>10.5</v>
       </c>
-      <c r="J98" s="1" t="n">
+      <c r="J98" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4410,7 +4434,7 @@
       <c r="I99" t="n">
         <v>-40.8</v>
       </c>
-      <c r="J99" s="1" t="n">
+      <c r="J99" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4450,7 +4474,7 @@
       <c r="I100" t="n">
         <v>2.2</v>
       </c>
-      <c r="J100" s="1" t="n">
+      <c r="J100" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4490,7 +4514,7 @@
       <c r="I101" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="J101" s="1" t="n">
+      <c r="J101" s="2" t="n">
         <v>46296.34375</v>
       </c>
     </row>
@@ -4530,7 +4554,7 @@
       <c r="I102" t="n">
         <v>11</v>
       </c>
-      <c r="J102" s="1" t="n">
+      <c r="J102" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4570,7 +4594,7 @@
       <c r="I103" t="n">
         <v>-11.1</v>
       </c>
-      <c r="J103" s="1" t="n">
+      <c r="J103" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4610,7 +4634,7 @@
       <c r="I104" t="n">
         <v>7.8</v>
       </c>
-      <c r="J104" s="1" t="n">
+      <c r="J104" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4650,7 +4674,7 @@
       <c r="I105" t="n">
         <v>1.8</v>
       </c>
-      <c r="J105" s="1" t="n">
+      <c r="J105" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4690,7 +4714,7 @@
       <c r="I106" t="n">
         <v>9</v>
       </c>
-      <c r="J106" s="1" t="n">
+      <c r="J106" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4730,7 +4754,7 @@
       <c r="I107" t="n">
         <v>14.2</v>
       </c>
-      <c r="J107" s="1" t="n">
+      <c r="J107" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4770,7 +4794,7 @@
       <c r="I108" t="n">
         <v>17.7</v>
       </c>
-      <c r="J108" s="1" t="n">
+      <c r="J108" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4810,7 +4834,7 @@
       <c r="I109" t="n">
         <v>0.3</v>
       </c>
-      <c r="J109" s="1" t="n">
+      <c r="J109" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4850,7 +4874,7 @@
       <c r="I110" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="J110" s="1" t="n">
+      <c r="J110" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4890,7 +4914,7 @@
       <c r="I111" t="n">
         <v>0.3</v>
       </c>
-      <c r="J111" s="1" t="n">
+      <c r="J111" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4930,7 +4954,7 @@
       <c r="I112" t="n">
         <v>10.1</v>
       </c>
-      <c r="J112" s="1" t="n">
+      <c r="J112" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -4970,7 +4994,7 @@
       <c r="I113" t="n">
         <v>-0.2</v>
       </c>
-      <c r="J113" s="1" t="n">
+      <c r="J113" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5010,7 +5034,7 @@
       <c r="I114" t="n">
         <v>22.8</v>
       </c>
-      <c r="J114" s="1" t="n">
+      <c r="J114" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5050,7 +5074,7 @@
       <c r="I115" t="n">
         <v>11.8</v>
       </c>
-      <c r="J115" s="1" t="n">
+      <c r="J115" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5090,7 +5114,7 @@
       <c r="I116" t="n">
         <v>20.5</v>
       </c>
-      <c r="J116" s="1" t="n">
+      <c r="J116" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5130,7 +5154,7 @@
       <c r="I117" t="n">
         <v>-6.9</v>
       </c>
-      <c r="J117" s="1" t="n">
+      <c r="J117" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5170,7 +5194,7 @@
       <c r="I118" t="n">
         <v>0.4</v>
       </c>
-      <c r="J118" s="1" t="n">
+      <c r="J118" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5210,7 +5234,7 @@
       <c r="I119" t="n">
         <v>-3.5</v>
       </c>
-      <c r="J119" s="1" t="n">
+      <c r="J119" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5250,7 +5274,7 @@
       <c r="I120" t="n">
         <v>11.5</v>
       </c>
-      <c r="J120" s="1" t="n">
+      <c r="J120" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5290,7 +5314,7 @@
       <c r="I121" t="n">
         <v>-5.3</v>
       </c>
-      <c r="J121" s="1" t="n">
+      <c r="J121" s="2" t="n">
         <v>46296.34583333333</v>
       </c>
     </row>
@@ -5330,7 +5354,7 @@
       <c r="I122" t="n">
         <v>-10.6</v>
       </c>
-      <c r="J122" s="1" t="n">
+      <c r="J122" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5370,7 +5394,7 @@
       <c r="I123" t="n">
         <v>2.5</v>
       </c>
-      <c r="J123" s="1" t="n">
+      <c r="J123" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5410,7 +5434,7 @@
       <c r="I124" t="n">
         <v>0.8</v>
       </c>
-      <c r="J124" s="1" t="n">
+      <c r="J124" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5445,12 +5469,12 @@
         <v>91.59999999999999</v>
       </c>
       <c r="H125" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I125" t="n">
         <v>-15.5</v>
       </c>
-      <c r="J125" s="1" t="n">
+      <c r="J125" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5490,7 +5514,7 @@
       <c r="I126" t="n">
         <v>11.2</v>
       </c>
-      <c r="J126" s="1" t="n">
+      <c r="J126" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5530,7 +5554,7 @@
       <c r="I127" t="n">
         <v>-0.5</v>
       </c>
-      <c r="J127" s="1" t="n">
+      <c r="J127" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5570,7 +5594,7 @@
       <c r="I128" t="n">
         <v>-13.2</v>
       </c>
-      <c r="J128" s="1" t="n">
+      <c r="J128" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5610,7 +5634,7 @@
       <c r="I129" t="n">
         <v>-2.3</v>
       </c>
-      <c r="J129" s="1" t="n">
+      <c r="J129" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5650,7 +5674,7 @@
       <c r="I130" t="n">
         <v>-0.2</v>
       </c>
-      <c r="J130" s="1" t="n">
+      <c r="J130" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5690,7 +5714,7 @@
       <c r="I131" t="n">
         <v>-26.2</v>
       </c>
-      <c r="J131" s="1" t="n">
+      <c r="J131" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5730,7 +5754,7 @@
       <c r="I132" t="n">
         <v>-22.5</v>
       </c>
-      <c r="J132" s="1" t="n">
+      <c r="J132" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5770,7 +5794,7 @@
       <c r="I133" t="n">
         <v>-20.4</v>
       </c>
-      <c r="J133" s="1" t="n">
+      <c r="J133" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5810,7 +5834,7 @@
       <c r="I134" t="n">
         <v>3.7</v>
       </c>
-      <c r="J134" s="1" t="n">
+      <c r="J134" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5850,7 +5874,7 @@
       <c r="I135" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="J135" s="1" t="n">
+      <c r="J135" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5890,7 +5914,7 @@
       <c r="I136" t="n">
         <v>-19.6</v>
       </c>
-      <c r="J136" s="1" t="n">
+      <c r="J136" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5930,7 +5954,7 @@
       <c r="I137" t="n">
         <v>-1.3</v>
       </c>
-      <c r="J137" s="1" t="n">
+      <c r="J137" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -5970,7 +5994,7 @@
       <c r="I138" t="n">
         <v>12.7</v>
       </c>
-      <c r="J138" s="1" t="n">
+      <c r="J138" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -6010,7 +6034,7 @@
       <c r="I139" t="n">
         <v>-5.7</v>
       </c>
-      <c r="J139" s="1" t="n">
+      <c r="J139" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -6050,7 +6074,7 @@
       <c r="I140" t="n">
         <v>-10.1</v>
       </c>
-      <c r="J140" s="1" t="n">
+      <c r="J140" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -6090,7 +6114,7 @@
       <c r="I141" t="n">
         <v>3.9</v>
       </c>
-      <c r="J141" s="1" t="n">
+      <c r="J141" s="2" t="n">
         <v>46296.34791666667</v>
       </c>
     </row>
@@ -6130,7 +6154,7 @@
       <c r="I142" t="n">
         <v>7.2</v>
       </c>
-      <c r="J142" s="1" t="n">
+      <c r="J142" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6170,7 +6194,7 @@
       <c r="I143" t="n">
         <v>-2.4</v>
       </c>
-      <c r="J143" s="1" t="n">
+      <c r="J143" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6210,7 +6234,7 @@
       <c r="I144" t="n">
         <v>-10.3</v>
       </c>
-      <c r="J144" s="1" t="n">
+      <c r="J144" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6250,7 +6274,7 @@
       <c r="I145" t="n">
         <v>15.4</v>
       </c>
-      <c r="J145" s="1" t="n">
+      <c r="J145" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6290,7 +6314,7 @@
       <c r="I146" t="n">
         <v>9.4</v>
       </c>
-      <c r="J146" s="1" t="n">
+      <c r="J146" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6330,7 +6354,7 @@
       <c r="I147" t="n">
         <v>5.5</v>
       </c>
-      <c r="J147" s="1" t="n">
+      <c r="J147" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6370,7 +6394,7 @@
       <c r="I148" t="n">
         <v>12.2</v>
       </c>
-      <c r="J148" s="1" t="n">
+      <c r="J148" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6410,7 +6434,7 @@
       <c r="I149" t="n">
         <v>-3.8</v>
       </c>
-      <c r="J149" s="1" t="n">
+      <c r="J149" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6450,7 +6474,7 @@
       <c r="I150" t="n">
         <v>0.6</v>
       </c>
-      <c r="J150" s="1" t="n">
+      <c r="J150" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6490,7 +6514,7 @@
       <c r="I151" t="n">
         <v>-2.1</v>
       </c>
-      <c r="J151" s="1" t="n">
+      <c r="J151" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6530,7 +6554,7 @@
       <c r="I152" t="n">
         <v>7</v>
       </c>
-      <c r="J152" s="1" t="n">
+      <c r="J152" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6570,7 +6594,7 @@
       <c r="I153" t="n">
         <v>24.1</v>
       </c>
-      <c r="J153" s="1" t="n">
+      <c r="J153" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6610,7 +6634,7 @@
       <c r="I154" t="n">
         <v>-23.2</v>
       </c>
-      <c r="J154" s="1" t="n">
+      <c r="J154" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6650,7 +6674,7 @@
       <c r="I155" t="n">
         <v>1.2</v>
       </c>
-      <c r="J155" s="1" t="n">
+      <c r="J155" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6690,7 +6714,7 @@
       <c r="I156" t="n">
         <v>-6.3</v>
       </c>
-      <c r="J156" s="1" t="n">
+      <c r="J156" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6730,7 +6754,7 @@
       <c r="I157" t="n">
         <v>23.8</v>
       </c>
-      <c r="J157" s="1" t="n">
+      <c r="J157" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6770,7 +6794,7 @@
       <c r="I158" t="n">
         <v>18.4</v>
       </c>
-      <c r="J158" s="1" t="n">
+      <c r="J158" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6810,7 +6834,7 @@
       <c r="I159" t="n">
         <v>16.9</v>
       </c>
-      <c r="J159" s="1" t="n">
+      <c r="J159" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6850,7 +6874,7 @@
       <c r="I160" t="n">
         <v>-15.8</v>
       </c>
-      <c r="J160" s="1" t="n">
+      <c r="J160" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6890,7 +6914,7 @@
       <c r="I161" t="n">
         <v>-23.2</v>
       </c>
-      <c r="J161" s="1" t="n">
+      <c r="J161" s="2" t="n">
         <v>46296.35</v>
       </c>
     </row>
@@ -6930,7 +6954,7 @@
       <c r="I162" t="n">
         <v>-6</v>
       </c>
-      <c r="J162" s="1" t="n">
+      <c r="J162" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -6970,7 +6994,7 @@
       <c r="I163" t="n">
         <v>23.7</v>
       </c>
-      <c r="J163" s="1" t="n">
+      <c r="J163" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7010,7 +7034,7 @@
       <c r="I164" t="n">
         <v>-19.3</v>
       </c>
-      <c r="J164" s="1" t="n">
+      <c r="J164" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7050,7 +7074,7 @@
       <c r="I165" t="n">
         <v>6.3</v>
       </c>
-      <c r="J165" s="1" t="n">
+      <c r="J165" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7090,7 +7114,7 @@
       <c r="I166" t="n">
         <v>1.5</v>
       </c>
-      <c r="J166" s="1" t="n">
+      <c r="J166" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7130,7 +7154,7 @@
       <c r="I167" t="n">
         <v>-29.1</v>
       </c>
-      <c r="J167" s="1" t="n">
+      <c r="J167" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7170,7 +7194,7 @@
       <c r="I168" t="n">
         <v>-13.2</v>
       </c>
-      <c r="J168" s="1" t="n">
+      <c r="J168" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7210,7 +7234,7 @@
       <c r="I169" t="n">
         <v>11.3</v>
       </c>
-      <c r="J169" s="1" t="n">
+      <c r="J169" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7250,7 +7274,7 @@
       <c r="I170" t="n">
         <v>-37.2</v>
       </c>
-      <c r="J170" s="1" t="n">
+      <c r="J170" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7290,7 +7314,7 @@
       <c r="I171" t="n">
         <v>-20.4</v>
       </c>
-      <c r="J171" s="1" t="n">
+      <c r="J171" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7330,7 +7354,7 @@
       <c r="I172" t="n">
         <v>17.9</v>
       </c>
-      <c r="J172" s="1" t="n">
+      <c r="J172" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7370,7 +7394,7 @@
       <c r="I173" t="n">
         <v>6.6</v>
       </c>
-      <c r="J173" s="1" t="n">
+      <c r="J173" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7410,7 +7434,7 @@
       <c r="I174" t="n">
         <v>10.9</v>
       </c>
-      <c r="J174" s="1" t="n">
+      <c r="J174" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7450,7 +7474,7 @@
       <c r="I175" t="n">
         <v>-2.4</v>
       </c>
-      <c r="J175" s="1" t="n">
+      <c r="J175" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7490,7 +7514,7 @@
       <c r="I176" t="n">
         <v>6.4</v>
       </c>
-      <c r="J176" s="1" t="n">
+      <c r="J176" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7530,7 +7554,7 @@
       <c r="I177" t="n">
         <v>-8.199999999999999</v>
       </c>
-      <c r="J177" s="1" t="n">
+      <c r="J177" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7570,7 +7594,7 @@
       <c r="I178" t="n">
         <v>-3.9</v>
       </c>
-      <c r="J178" s="1" t="n">
+      <c r="J178" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7610,7 +7634,7 @@
       <c r="I179" t="n">
         <v>2.7</v>
       </c>
-      <c r="J179" s="1" t="n">
+      <c r="J179" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7650,7 +7674,7 @@
       <c r="I180" t="n">
         <v>11.9</v>
       </c>
-      <c r="J180" s="1" t="n">
+      <c r="J180" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7690,7 +7714,7 @@
       <c r="I181" t="n">
         <v>34.7</v>
       </c>
-      <c r="J181" s="1" t="n">
+      <c r="J181" s="2" t="n">
         <v>46296.35208333333</v>
       </c>
     </row>
@@ -7730,7 +7754,7 @@
       <c r="I182" t="n">
         <v>33.3</v>
       </c>
-      <c r="J182" s="1" t="n">
+      <c r="J182" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -7770,7 +7794,7 @@
       <c r="I183" t="n">
         <v>-10</v>
       </c>
-      <c r="J183" s="1" t="n">
+      <c r="J183" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -7810,7 +7834,7 @@
       <c r="I184" t="n">
         <v>-25.8</v>
       </c>
-      <c r="J184" s="1" t="n">
+      <c r="J184" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -7850,7 +7874,7 @@
       <c r="I185" t="n">
         <v>1.8</v>
       </c>
-      <c r="J185" s="1" t="n">
+      <c r="J185" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -7890,7 +7914,7 @@
       <c r="I186" t="n">
         <v>-12.2</v>
       </c>
-      <c r="J186" s="1" t="n">
+      <c r="J186" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -7930,7 +7954,7 @@
       <c r="I187" t="n">
         <v>-4.5</v>
       </c>
-      <c r="J187" s="1" t="n">
+      <c r="J187" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -7970,7 +7994,7 @@
       <c r="I188" t="n">
         <v>2.5</v>
       </c>
-      <c r="J188" s="1" t="n">
+      <c r="J188" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8010,7 +8034,7 @@
       <c r="I189" t="n">
         <v>0.5</v>
       </c>
-      <c r="J189" s="1" t="n">
+      <c r="J189" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8050,7 +8074,7 @@
       <c r="I190" t="n">
         <v>4</v>
       </c>
-      <c r="J190" s="1" t="n">
+      <c r="J190" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8090,7 +8114,7 @@
       <c r="I191" t="n">
         <v>16.4</v>
       </c>
-      <c r="J191" s="1" t="n">
+      <c r="J191" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8130,7 +8154,7 @@
       <c r="I192" t="n">
         <v>-14.7</v>
       </c>
-      <c r="J192" s="1" t="n">
+      <c r="J192" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8170,7 +8194,7 @@
       <c r="I193" t="n">
         <v>-31.6</v>
       </c>
-      <c r="J193" s="1" t="n">
+      <c r="J193" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8210,7 +8234,7 @@
       <c r="I194" t="n">
         <v>4</v>
       </c>
-      <c r="J194" s="1" t="n">
+      <c r="J194" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8250,7 +8274,7 @@
       <c r="I195" t="n">
         <v>-9.199999999999999</v>
       </c>
-      <c r="J195" s="1" t="n">
+      <c r="J195" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8290,7 +8314,7 @@
       <c r="I196" t="n">
         <v>-15.2</v>
       </c>
-      <c r="J196" s="1" t="n">
+      <c r="J196" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8330,7 +8354,7 @@
       <c r="I197" t="n">
         <v>0.7</v>
       </c>
-      <c r="J197" s="1" t="n">
+      <c r="J197" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8370,7 +8394,7 @@
       <c r="I198" t="n">
         <v>-7</v>
       </c>
-      <c r="J198" s="1" t="n">
+      <c r="J198" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8410,7 +8434,7 @@
       <c r="I199" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="J199" s="1" t="n">
+      <c r="J199" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8450,7 +8474,7 @@
       <c r="I200" t="n">
         <v>-2.7</v>
       </c>
-      <c r="J200" s="1" t="n">
+      <c r="J200" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8490,7 +8514,7 @@
       <c r="I201" t="n">
         <v>-0.4</v>
       </c>
-      <c r="J201" s="1" t="n">
+      <c r="J201" s="2" t="n">
         <v>46296.35416666666</v>
       </c>
     </row>
@@ -8530,7 +8554,7 @@
       <c r="I202" t="n">
         <v>-3.1</v>
       </c>
-      <c r="J202" s="1" t="n">
+      <c r="J202" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8570,7 +8594,7 @@
       <c r="I203" t="n">
         <v>1.9</v>
       </c>
-      <c r="J203" s="1" t="n">
+      <c r="J203" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8610,7 +8634,7 @@
       <c r="I204" t="n">
         <v>12.8</v>
       </c>
-      <c r="J204" s="1" t="n">
+      <c r="J204" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8650,7 +8674,7 @@
       <c r="I205" t="n">
         <v>-7.3</v>
       </c>
-      <c r="J205" s="1" t="n">
+      <c r="J205" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8690,7 +8714,7 @@
       <c r="I206" t="n">
         <v>3</v>
       </c>
-      <c r="J206" s="1" t="n">
+      <c r="J206" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8730,7 +8754,7 @@
       <c r="I207" t="n">
         <v>2.2</v>
       </c>
-      <c r="J207" s="1" t="n">
+      <c r="J207" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8770,7 +8794,7 @@
       <c r="I208" t="n">
         <v>12.8</v>
       </c>
-      <c r="J208" s="1" t="n">
+      <c r="J208" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8810,7 +8834,7 @@
       <c r="I209" t="n">
         <v>-10.7</v>
       </c>
-      <c r="J209" s="1" t="n">
+      <c r="J209" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8850,7 +8874,7 @@
       <c r="I210" t="n">
         <v>37.4</v>
       </c>
-      <c r="J210" s="1" t="n">
+      <c r="J210" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8890,7 +8914,7 @@
       <c r="I211" t="n">
         <v>-11.2</v>
       </c>
-      <c r="J211" s="1" t="n">
+      <c r="J211" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8930,7 +8954,7 @@
       <c r="I212" t="n">
         <v>-8.699999999999999</v>
       </c>
-      <c r="J212" s="1" t="n">
+      <c r="J212" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -8970,7 +8994,7 @@
       <c r="I213" t="n">
         <v>-10.4</v>
       </c>
-      <c r="J213" s="1" t="n">
+      <c r="J213" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9010,7 +9034,7 @@
       <c r="I214" t="n">
         <v>-0.3</v>
       </c>
-      <c r="J214" s="1" t="n">
+      <c r="J214" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9050,7 +9074,7 @@
       <c r="I215" t="n">
         <v>-10.6</v>
       </c>
-      <c r="J215" s="1" t="n">
+      <c r="J215" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9090,7 +9114,7 @@
       <c r="I216" t="n">
         <v>-1.8</v>
       </c>
-      <c r="J216" s="1" t="n">
+      <c r="J216" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9130,7 +9154,7 @@
       <c r="I217" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="J217" s="1" t="n">
+      <c r="J217" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9170,7 +9194,7 @@
       <c r="I218" t="n">
         <v>-12.1</v>
       </c>
-      <c r="J218" s="1" t="n">
+      <c r="J218" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9210,7 +9234,7 @@
       <c r="I219" t="n">
         <v>8.5</v>
       </c>
-      <c r="J219" s="1" t="n">
+      <c r="J219" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9250,7 +9274,7 @@
       <c r="I220" t="n">
         <v>-9.6</v>
       </c>
-      <c r="J220" s="1" t="n">
+      <c r="J220" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9290,7 +9314,7 @@
       <c r="I221" t="n">
         <v>-5.3</v>
       </c>
-      <c r="J221" s="1" t="n">
+      <c r="J221" s="2" t="n">
         <v>46296.35625</v>
       </c>
     </row>
@@ -9330,7 +9354,7 @@
       <c r="I222" t="n">
         <v>0.3</v>
       </c>
-      <c r="J222" s="1" t="n">
+      <c r="J222" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9370,7 +9394,7 @@
       <c r="I223" t="n">
         <v>6.2</v>
       </c>
-      <c r="J223" s="1" t="n">
+      <c r="J223" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9410,7 +9434,7 @@
       <c r="I224" t="n">
         <v>7.7</v>
       </c>
-      <c r="J224" s="1" t="n">
+      <c r="J224" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9450,7 +9474,7 @@
       <c r="I225" t="n">
         <v>-0.9</v>
       </c>
-      <c r="J225" s="1" t="n">
+      <c r="J225" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9490,7 +9514,7 @@
       <c r="I226" t="n">
         <v>30</v>
       </c>
-      <c r="J226" s="1" t="n">
+      <c r="J226" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9530,7 +9554,7 @@
       <c r="I227" t="n">
         <v>1.2</v>
       </c>
-      <c r="J227" s="1" t="n">
+      <c r="J227" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9570,7 +9594,7 @@
       <c r="I228" t="n">
         <v>1.1</v>
       </c>
-      <c r="J228" s="1" t="n">
+      <c r="J228" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9610,7 +9634,7 @@
       <c r="I229" t="n">
         <v>21.4</v>
       </c>
-      <c r="J229" s="1" t="n">
+      <c r="J229" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9650,7 +9674,7 @@
       <c r="I230" t="n">
         <v>-15.1</v>
       </c>
-      <c r="J230" s="1" t="n">
+      <c r="J230" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9690,7 +9714,7 @@
       <c r="I231" t="n">
         <v>21.4</v>
       </c>
-      <c r="J231" s="1" t="n">
+      <c r="J231" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9730,7 +9754,7 @@
       <c r="I232" t="n">
         <v>-0.7</v>
       </c>
-      <c r="J232" s="1" t="n">
+      <c r="J232" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9770,7 +9794,7 @@
       <c r="I233" t="n">
         <v>-13.3</v>
       </c>
-      <c r="J233" s="1" t="n">
+      <c r="J233" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9810,7 +9834,7 @@
       <c r="I234" t="n">
         <v>-15.7</v>
       </c>
-      <c r="J234" s="1" t="n">
+      <c r="J234" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9850,7 +9874,7 @@
       <c r="I235" t="n">
         <v>5.5</v>
       </c>
-      <c r="J235" s="1" t="n">
+      <c r="J235" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9890,7 +9914,7 @@
       <c r="I236" t="n">
         <v>-11.6</v>
       </c>
-      <c r="J236" s="1" t="n">
+      <c r="J236" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9930,7 +9954,7 @@
       <c r="I237" t="n">
         <v>15.5</v>
       </c>
-      <c r="J237" s="1" t="n">
+      <c r="J237" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -9970,7 +9994,7 @@
       <c r="I238" t="n">
         <v>-4.7</v>
       </c>
-      <c r="J238" s="1" t="n">
+      <c r="J238" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -10010,7 +10034,7 @@
       <c r="I239" t="n">
         <v>-19.9</v>
       </c>
-      <c r="J239" s="1" t="n">
+      <c r="J239" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -10050,7 +10074,7 @@
       <c r="I240" t="n">
         <v>-18.1</v>
       </c>
-      <c r="J240" s="1" t="n">
+      <c r="J240" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>
@@ -10090,7 +10114,7 @@
       <c r="I241" t="n">
         <v>12.1</v>
       </c>
-      <c r="J241" s="1" t="n">
+      <c r="J241" s="2" t="n">
         <v>46296.35833333333</v>
       </c>
     </row>

</xml_diff>